<commit_message>
updated datasets and bertopic pipline
</commit_message>
<xml_diff>
--- a/ML_models/component02/data/news.xlsx
+++ b/ML_models/component02/data/news.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Research\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9D1DE4E-21E1-4A82-9C95-A5231D6D4E96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5B9C050-B4C5-43B9-B41A-9F1A090CB4DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{0009C542-81AE-4BF4-B856-6D3C58BA2BF2}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="38">
   <si>
     <t>date</t>
   </si>
@@ -44,9 +44,6 @@
     <t>record_id</t>
   </si>
   <si>
-    <t>source</t>
-  </si>
-  <si>
     <t>location</t>
   </si>
   <si>
@@ -56,27 +53,18 @@
     <t>2025.10.05</t>
   </si>
   <si>
-    <t>Hiru news</t>
-  </si>
-  <si>
     <t>Narangala</t>
   </si>
   <si>
     <t>2023.12.02</t>
   </si>
   <si>
-    <t>Ada derana</t>
-  </si>
-  <si>
     <t>Hanthana</t>
   </si>
   <si>
     <t>2025.06.29</t>
   </si>
   <si>
-    <t>DailyNews</t>
-  </si>
-  <si>
     <t>2016.05.26</t>
   </si>
   <si>
@@ -95,33 +83,48 @@
     <t>Sigirya</t>
   </si>
   <si>
-    <t>Newsfirst</t>
-  </si>
-  <si>
     <t>2022.02.22</t>
   </si>
   <si>
-    <t>The Sunday times</t>
-  </si>
-  <si>
     <t>Pidurangala</t>
   </si>
   <si>
-    <t>Hikers trapped on Narangala mountain after heavy rain and wind:22 members of three local youth groups who set out to climb the Narangala Mountain in Hali-Ela are now stranded on the summit following the sudden onset of torrential rain and strong winds this afternoon (4 October), according to the Disaster Management Centre.
+    <t>2025.12.19</t>
+  </si>
+  <si>
+    <t>Little Adam's peak</t>
+  </si>
+  <si>
+    <t>2026.01.10</t>
+  </si>
+  <si>
+    <t>2024.08.02</t>
+  </si>
+  <si>
+    <t>2025.11.25</t>
+  </si>
+  <si>
+    <t>Pettigala</t>
+  </si>
+  <si>
+    <t>2019.04.28</t>
+  </si>
+  <si>
+    <t>Hiru news: Hikers trapped on Narangala mountain after heavy rain and wind:22 members of three local youth groups who set out to climb the Narangala Mountain in Hali-Ela are now stranded on the summit following the sudden onset of torrential rain and strong winds this afternoon (4 October), according to the Disaster Management Centre.
 The Kandegedara Police stated that officials from the station, along with an Army team from the Badulla Eladaluwa Army Camp, have been dispatched to the mountain to rescue the 22 stranded individuals safely. The groups, who are residents of the Negombo area, were attempting to climb Narangala Mountain this afternoon.Reports indicate that the sudden heavy rain and severe wind tore away their tents, leaving them stranded on the summit.Police confirmed that the groups are in distress due to the wind and intense cold. Authorities are currently maintaining contact with the hikers via their mobile phones and are working to rescue them as quickly as possible.</t>
   </si>
   <si>
-    <t>At least 180 university students rescued after getting lost in Hanthana mountains: A group of at least 180 university students, who were stranded in the Hanthana mountain range during a hike, have been rescued.They were found during a search and rescue operation jointly carried out by the army and police. According to reports, the group comprised students of the Kelaniya University’s Faculty of Medicine in Ragama.The thick fog in the area had initially made it difficult for the rescuers to locate the stranded students.</t>
-  </si>
-  <si>
-    <t>Army Rescues Young Group Stranded in Hanthana: Eight children and young adults aged between 12 and 24 years, who had gone hiking in the Hanthana mountain range in Kandy on June 28, became stranded due to adverse weather conditions.Upon receiving the information, a rescue operation was promptly launched by personnel from the 2nd Sri Lanka Lions Volunteer Regiment of the Sri Lanka Army. After an intense 8-hour operation, Army troops successfully located and rescued all eight individuals. They were subsequently handed over to the Thalathuoya Police and later referred to the Peradeniya General Hospital for medical observation. Authorities have urged hikers and tourists to take necessary precautions and monitor weather alerts before trekking in mountainous areas.</t>
-  </si>
-  <si>
-    <t>Crevice Appears on Hanthana Mountain: The Hanthaana Conservation Organization states that a crevice has appeared on the mountain side near the 7th Mile Post on the Kandy Uduwela road.
+    <t>Ada derana: At least 180 university students rescued after getting lost in Hanthana mountains: A group of at least 180 university students, who were stranded in the Hanthana mountain range during a hike, have been rescued.They were found during a search and rescue operation jointly carried out by the army and police. According to reports, the group comprised students of the Kelaniya University’s Faculty of Medicine in Ragama.The thick fog in the area had initially made it difficult for the rescuers to locate the stranded students.</t>
+  </si>
+  <si>
+    <t>DailyNews: Army Rescues Young Group Stranded in Hanthana: Eight children and young adults aged between 12 and 24 years, who had gone hiking in the Hanthana mountain range in Kandy on June 28, became stranded due to adverse weather conditions.Upon receiving the information, a rescue operation was promptly launched by personnel from the 2nd Sri Lanka Lions Volunteer Regiment of the Sri Lanka Army. After an intense 8-hour operation, Army troops successfully located and rescued all eight individuals. They were subsequently handed over to the Thalathuoya Police and later referred to the Peradeniya General Hospital for medical observation. Authorities have urged hikers and tourists to take necessary precautions and monitor weather alerts before trekking in mountainous areas.</t>
+  </si>
+  <si>
+    <t>Hiru news: Crevice Appears on Hanthana Mountain: The Hanthaana Conservation Organization states that a crevice has appeared on the mountain side near the 7th Mile Post on the Kandy Uduwela road.
 Organization’s Secretary Amith Senanayake said that this crevice could lead to a landslide.</t>
   </si>
   <si>
-    <t>Army rescues missing hiker from Hanthana Mountain Range: An individual who had gone to climb “Katusu Konda” in the Hanthana Mountain Range and went missing has been successfully rescued by the Sri Lanka Army.
+    <t>Ada derana: Army rescues missing hiker from Hanthana Mountain Range: An individual who had gone to climb “Katusu Konda” in the Hanthana Mountain Range and went missing has been successfully rescued by the Sri Lanka Army.
 The Army stated that he was rescued during a special operation carried out this morning (13).
 Troops from the 2nd (Volunteer) Battalion of the Sri Lanka Sinha Regiment, belonging to the 111 Infantry Brigade of the army, took part in this operation.
 According to information received from the Kandy Police, a team consisting of two Army officers and eight soldiers commenced the rescue mission yesterday (12) at around 6:40 p.m.
@@ -129,16 +132,35 @@
 Accordingly, at around 7:45 a.m. today (13), the Army personnel were able to locate the missing person unharmed.</t>
   </si>
   <si>
-    <t>Wasps rise again at Sigiriya:Wasps attacked tourists again this morning (February 13), reports the Adaderana correspondent at the historic Rock Fortress of Sigiriya. Eighteen persons, mostly foreign tourists were stung by the swarming wasps, he says.
+    <t>Ada derana: Wasps rise again at Sigiriya:Wasps attacked tourists again this morning (February 13), reports the Adaderana correspondent at the historic Rock Fortress of Sigiriya. Eighteen persons, mostly foreign tourists were stung by the swarming wasps, he says.
 On several occasions in the recent past too the wasps who have made their nesting place on the sides of the rock have attacked tourists climbing the citadel in the sky built by King Kasyappa.</t>
   </si>
   <si>
-    <t>22 Tourists Hospitalized After Wasp Attack at Sigiriya: COLOMBO (News 1st); 22 foreign tourists visiting the historic Sigiriya rock fortress in Sri Lanka were hospitalized after being stung by wasps. 
+    <t>Newsfirst: 22 Tourists Hospitalized After Wasp Attack at Sigiriya: COLOMBO (News 1st); 22 foreign tourists visiting the historic Sigiriya rock fortress in Sri Lanka were hospitalized after being stung by wasps. 
 The incident occurred when a part of a wasp hive collapsed due to high wind conditions, leading to the unfortunate stings.Professor Gamini Ranasinghe, the Director General of the Central Cultural Fund, confirmed the cause of the incident and announced that the Sigiriya premises had to be temporarily closed to ensure the safety of visitors.The situation has been brought under control, and Sigiriya has now reopened for tourists.</t>
   </si>
   <si>
-    <t>Pidurangala’s pachyderm problem needs “sustainable solution”: The death of a foreign tourist due to a wild elephant attack at Pidurangala in Sigiriya last week points to the lack of personnel and resources within the Wildlife Department as well as a lack of tourist awareness of possible wild elephant encounters after dark in the area, experts said. In the vicinity of Pidurangala, frequented daily by more than 5,000 tourists as well as other commuters, the Wildlife Department does not have the human resources to take effective measures against the human-elephant conflict, said Sigiriya Tourist Police OIC Inspector Dissanayake, who investigated the death of Hungarian tourist Professor Joe Anton, who had visited the Pidurangala rock with his wife last week.
+    <t>The Sunday times: Pidurangala’s pachyderm problem needs “sustainable solution”: The death of a foreign tourist due to a wild elephant attack at Pidurangala in Sigiriya last week points to the lack of personnel and resources within the Wildlife Department as well as a lack of tourist awareness of possible wild elephant encounters after dark in the area, experts said. In the vicinity of Pidurangala, frequented daily by more than 5,000 tourists as well as other commuters, the Wildlife Department does not have the human resources to take effective measures against the human-elephant conflict, said Sigiriya Tourist Police OIC Inspector Dissanayake, who investigated the death of Hungarian tourist Professor Joe Anton, who had visited the Pidurangala rock with his wife last week.
 Tourists share the responsibility of their actions equally for visiting the area after dark, against advice not to do so,” the OIC emphasised. Inspector Dissanayake said that while hotel and tourist accommodation owners warn tourists against walking in the area after darkness, this is not communicated rigorously enough. While the Sigiriya tourist site is well-lit and secure from elephants, Pidurangala is part of a wildlife sanctuary and not cleared of wild elephants. According to the UK-based Guardian, the human-elephant conflict in Sri Lanka is among the most severe in the world, causing approximately 400-470 elephant deaths and 100-180 human fatalities annually.</t>
+  </si>
+  <si>
+    <t>Newsfirst: Woman Survives Cliff Plunge At Little Adam's Peak: COLOMBO (News 1st); A British woman narrowly escaped tragedy yesterday afternoon after falling nearly 100 feet down a cliff while visiting the picturesque Little Adam's Peak in the Ella Police Division. The incident occurred in the 3rd Mile Post area, a popular vantage point for hikers and nature lovers. According to local authorities, the woman had been admiring the breathtaking views when she accidentally slipped and plunged into the ravine.Emergency rescue teams rushed to the scene and carried out a challenging operation to bring her to safety. Despite the severity of the fall, she was successfully rescued and transported to Badulla Hospital for treatment. Mini Sri Pada, often called the “Little Adam’s Peak,” is a major tourist attraction in Ella, drawing hundreds of visitors daily for its panoramic views and serene hiking trails.</t>
+  </si>
+  <si>
+    <t>Daily mirror: Colombo, January. 10 (Daily Mirror) - A foreign tourist child was rescued today after falling from a steep cliff at Little Adam’s Peak, officials said. The child is believed to have slipped while trying to take a selfie at the popular viewpoint, falling nearly 100 feet down the slope. The First Responder Rope Rescue Team from the Flying Ravana Adventure Park was immediately dispatched and carried out an emergency rescue amid difficult terrain.Rescuers successfully reached the child and brought her to safety. Witnesses said the child’s mother was visibly shaken during the operation but was relieved after her daughter was safely recovered. In light of the incident, authorities have urged visitors to exercise caution at high-risk areas of tourist attractions.</t>
+  </si>
+  <si>
+    <t>Ada derana: British woman injured after falling from Little Adam’s Peak: A female foreign tourist has been injured after falling from Little Adam’s Peak in Ella.Police said that the accident had occurred yesterday (01) during a visit to the tourist attraction.
+The 33-year-old British national has been rescued and rushed to Badulla Teaching Hospital by the Tourist Police with the assistance of a group of local tourists. She has sustained injuries to her right leg and is currently receiving treatment at the hospital, according to hospital sources.</t>
+  </si>
+  <si>
+    <t>Daily news: Foreign tourist’s child rescued after fall at Little Adam’s Peak:A foreign tourist child was rescued today (10) after falling from a steep cliff at the popular Little Adam’s Peak tourist attraction, authorities confirmed.The child reportedly fell nearly 100 feet while attempting to take a selfie near the edge of the cliff. Following the incident, the Flying Ravana Adventure Park’s first responder rope rescue team was immediately deployed to the location and carried out an emergency rescue operation.Despite the challenging terrain, rescuers successfully reached the child and brought her to safety.Witnesses said the child’s mother was visibly emotional and expressed immense relief after her daughter was rescued without serious harm.Authorities have once again urged both local and foreign tourists to exercise extreme caution when taking photographs or selfies at elevated tourist sites, particularly in areas close to cliffs and steep drop-offs.</t>
+  </si>
+  <si>
+    <t>Hiru news: Landslide risk forces Pettigala evacuations: Approximately 30 people in the Pettigala area of Balangoda were relocated to safe places due to a landslide risk.The District Disaster Management Centre stated the residents were evacuated because signs of a landslide emerged in the Pettigala area due to the heavy rainfall persisting in the region for several days.Meanwhile, a landslide in Kumbalwela, Bandarawela, damaged a house. Separately, a landslide in the Panwilahena area of Udugama damaged four houses.With the continuing rain, the landslide warnings remain active for 11 districts. The National Building Research Organisation stated the warning is in effect for the districts of Colombo, Kalutara, Galle, Matara, Hambantota, Kandy, Matale, Nuwara Eliya, Ratnapura, Kegalle, and Kurunegala.Additionally, due to the rain, the Kamburupitiya-Mulatiana road is flooded in the Makandura area. Reports indicate only heavy vehicles are able to use this road.</t>
+  </si>
+  <si>
+    <t>Newsfirst: Landslide threat: COLOMBO (News 1st) - Seventy-three people from 23 families from the Pettigala Estate, Balangoda were evacuated due to a landslide warning. Hemantha Bandara, Divisional Secretary, Balangoda,  said that the evacuated persons have been accommodated at the Pettigala school playground.</t>
   </si>
 </sst>
 </file>
@@ -513,16 +535,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{516B63CE-C943-4D19-B020-114EB7DA4A8D}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="13" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="20.5546875" customWidth="1"/>
-    <col min="5" max="5" width="66.77734375" customWidth="1"/>
+    <col min="3" max="3" width="20.5546875" customWidth="1"/>
+    <col min="4" max="4" width="66.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -532,150 +553,208 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="201.6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:4" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="D2" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="144" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="144" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" t="s">
-        <v>10</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="201.6" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="129.6" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8" t="s">
-        <v>18</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="273.60000000000002" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="288" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="172.8" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="144" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
         <v>20</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="187.2" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="187.2" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
         <v>21</v>
       </c>
-      <c r="D9" t="s">
+      <c r="C14" t="s">
         <v>22</v>
       </c>
-      <c r="E9" s="1" t="s">
-        <v>30</v>
+      <c r="D14" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>